<commit_message>
Move Hoopa to a Solaceon Ruins dead end and Eternatus to Victory Road B1F
Hoopa leaves Room 7 (Jirachi's) for Room 6's north-west dead end (2, 3);
Eternatus leaves Turnback Cave's Giratina room for Victory Road B1F's TM59
island (14, 19). Both maps get their own script archives. The Archivist's
hints now name the new places, Enamorus's and Yveltal's included.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sispid5Qo8kvdYnx3crKZR
</commit_message>
<xml_diff>
--- a/docs/StaticEncounters.xlsx
+++ b/docs/StaticEncounters.xlsx
@@ -190,10 +190,10 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1505,12 +1505,12 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Solaceon Ruins Room 7</t>
+          <t>Solaceon Ruins Room 6, north-west dead end</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>(5, 4)</t>
+          <t>(2, 3)</t>
         </is>
       </c>
       <c r="G22" s="4" t="n">
@@ -1521,14 +1521,14 @@
           <t>Prison Bottle in the bag</t>
         </is>
       </c>
-      <c r="I22" s="9" t="inlineStr">
-        <is>
-          <t>Clash</t>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>Directly below Jirachi (5, 3) in one small room. Move one</t>
+          <t>MOVED 2026-10-24 from Room 7 (5, 4), below Jirachi. The dead end holds nothing else</t>
         </is>
       </c>
     </row>
@@ -2273,12 +2273,12 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Turnback Cave, Giratina's room</t>
+          <t>Victory Road B1F, the TM59 island (Surf)</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>(8, 13)</t>
+          <t>(14, 19)</t>
         </is>
       </c>
       <c r="G38" s="4" t="n">
@@ -2289,14 +2289,14 @@
           <t>Zacian and Zamazenta caught</t>
         </is>
       </c>
-      <c r="I38" s="9" t="inlineStr">
-        <is>
-          <t>Clash</t>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>Giratina returns to this room after a Hall of Fame. Move Eternatus</t>
+          <t>MOVED 2026-10-24 from Turnback Cave's Giratina room (8, 13). Shares the island with the TM59 ball (13, 18); Moltres's portal is in a 1F room</t>
         </is>
       </c>
     </row>
@@ -3181,14 +3181,14 @@
           <t>Story; after a Hall of Fame if not caught</t>
         </is>
       </c>
-      <c r="I57" s="9" t="inlineStr">
-        <is>
-          <t>Clash</t>
+      <c r="I57" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
-          <t>Shares its room with Eternatus (8, 13)</t>
+          <t>Eternatus moved out on 2026-10-24</t>
         </is>
       </c>
     </row>
@@ -3973,14 +3973,14 @@
           <t>Three wishes granted</t>
         </is>
       </c>
-      <c r="I74" s="9" t="inlineStr">
-        <is>
-          <t>Clash</t>
+      <c r="I74" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
-          <t>Directly above Hoopa (5, 4)</t>
+          <t>Hoopa moved to Room 6 on 2026-10-24</t>
         </is>
       </c>
     </row>
@@ -4932,44 +4932,44 @@
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>Solaceon Ruins Room 7</t>
+          <t>Solaceon Ruins</t>
         </is>
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>Hoopa (5, 4); Jirachi (5, 3)</t>
-        </is>
-      </c>
-      <c r="C3" s="16" t="inlineStr">
-        <is>
-          <t>Clash</t>
+          <t>Jirachi (Room 7, 5, 3); Hoopa (Room 6 north-west dead end, 2, 3)</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="D3" s="15" t="inlineStr">
         <is>
-          <t>Move one, e.g. Hoopa to another Unown room</t>
+          <t>Settled 2026-10-24: Hoopa moved to Room 6</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>Turnback Cave, Giratina's room</t>
+          <t>Turnback Cave / Victory Road B1F</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>Eternatus (8, 13); Giratina (after a Hall of Fame)</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="inlineStr">
-        <is>
-          <t>Clash</t>
+          <t>Giratina (its room); Eternatus (Victory Road B1F, 14, 19)</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>Move Eternatus</t>
+          <t>Settled 2026-10-24: Eternatus moved to Victory Road B1F</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
           <t>Kyurem (Iceberg doorway room, 7, 5); Regice's ruins; Cosmog (35, 21); Articuno portal (to place); Kyogre (B1F); Totem Kommo-o (6F)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5050,7 +5050,7 @@
           <t>Virizion (80, 10); Xerneas (70, 14); Totem Vikavolt (22, 68); Celebi portals (to place)</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5072,7 +5072,7 @@
           <t>Totem Marowak (3, 4); Ho-Oh portal (to place)</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5094,7 +5094,7 @@
           <t>Totem Mimikyu (26, 10); Marshadow (21, 9)</t>
         </is>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5116,7 +5116,7 @@
           <t>Totem Togedemaru (10, 7); Victini (2, 7); Electric Master (4, 3)</t>
         </is>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5138,7 +5138,7 @@
           <t>Totem Salazzle (181, 585); Chi-Yu (180, 593) and stakes 7–8</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5160,7 +5160,7 @@
           <t>Totem Ribombee (18, 43); Tapu Bulu (24, 36)</t>
         </is>
       </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="C13" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5182,7 +5182,7 @@
           <t>Totem Araquanid (713, 826); Suicune (689, 826)</t>
         </is>
       </c>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5204,7 +5204,7 @@
           <t>Tapu Fini (716, 345); Wyver (717, 346)</t>
         </is>
       </c>
-      <c r="C15" s="17" t="inlineStr">
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5226,7 +5226,7 @@
           <t>Diancie (2, 22); Meltan (5, 20); Melmetal (5, 24)</t>
         </is>
       </c>
-      <c r="C16" s="17" t="inlineStr">
+      <c r="C16" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5248,7 +5248,7 @@
           <t>Tapu Lele (13, 12); Cresselia then Latias/Latios (16, 15)</t>
         </is>
       </c>
-      <c r="C17" s="17" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5270,7 +5270,7 @@
           <t>Koraidon (29, 36); Miraidon (27, 37); Terapagos (30, 34)</t>
         </is>
       </c>
-      <c r="C18" s="17" t="inlineStr">
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5292,7 +5292,7 @@
           <t>Zygarde (B1F 21, 4); Necrozma (1F 70, 9); Mira's quest</t>
         </is>
       </c>
-      <c r="C19" s="17" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5314,7 +5314,7 @@
           <t>Magearna (11, 13); Volkner</t>
         </is>
       </c>
-      <c r="C20" s="17" t="inlineStr">
+      <c r="C20" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5336,7 +5336,7 @@
           <t>Kubfu (13, 17); the Gym puzzle</t>
         </is>
       </c>
-      <c r="C21" s="17" t="inlineStr">
+      <c r="C21" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5358,7 +5358,7 @@
           <t>Calyrex (461, 527); the elder, the ruins path</t>
         </is>
       </c>
-      <c r="C22" s="17" t="inlineStr">
+      <c r="C22" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5380,7 +5380,7 @@
           <t>Meloetta (27, 8)</t>
         </is>
       </c>
-      <c r="C23" s="17" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -5402,7 +5402,7 @@
           <t>Enamorus (912, 535); Pecharunt (898, 526); Shaymin tablet (908, 491)</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C24" s="17" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -5424,7 +5424,7 @@
           <t>Yveltal (813, 426); Gene (827, 438)</t>
         </is>
       </c>
-      <c r="C25" s="18" t="inlineStr">
+      <c r="C25" s="17" t="inlineStr">
         <is>
           <t>None</t>
         </is>

</xml_diff>

<commit_message>
Move Landorus out of the Rock Peak Ruins room to Route 228's sand field
Landorus now waits at the north end of Route 228's first sand field
(782, 323); the ruins doorway room keeps Regidrago. The Archivist's hint
points to the sands of Route 228.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sispid5Qo8kvdYnx3crKZR
</commit_message>
<xml_diff>
--- a/docs/StaticEncounters.xlsx
+++ b/docs/StaticEncounters.xlsx
@@ -1217,12 +1217,12 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Route 228, Rock Peak Ruins chamber</t>
+          <t>Route 228, north end of the first sand field</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>(7, 5)</t>
+          <t>(782, 323)</t>
         </is>
       </c>
       <c r="G16" s="4" t="n">
@@ -1233,14 +1233,14 @@
           <t>Tornadus and Thundurus in the party</t>
         </is>
       </c>
-      <c r="I16" s="9" t="inlineStr">
-        <is>
-          <t>Clash</t>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>Two tiles from Regidrago (5, 6), in Regirock's puzzle chamber. Check the statue and dots</t>
+          <t>MOVED 2026-10-24 from the Rock Peak Ruins doorway room (7, 5). Ace Trainer Jose (779, 325) looks west/east on another row</t>
         </is>
       </c>
     </row>
@@ -2573,14 +2573,14 @@
           <t>Regirock, Regice, Registeel in the party</t>
         </is>
       </c>
-      <c r="I44" s="9" t="inlineStr">
-        <is>
-          <t>Clash</t>
+      <c r="I44" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>Two tiles from Landorus (7, 5), in Regirock's puzzle chamber</t>
+          <t>Landorus moved outside on 2026-10-24</t>
         </is>
       </c>
     </row>
@@ -3700,7 +3700,7 @@
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>Rock Peak: Landorus and Regidrago in the chamber. Iceberg: Kyurem's doorway room</t>
+          <t>Iceberg: Kyurem's doorway room. Rock Peak is settled (Landorus moved)</t>
         </is>
       </c>
     </row>
@@ -4976,22 +4976,22 @@
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>Route 228, Rock Peak Ruins chamber</t>
+          <t>Route 228</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>Landorus (7, 5); Regidrago (5, 6); Regirock's statue and dots</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>Clash</t>
+          <t>Landorus (782, 323, outside); Regidrago (Rock Peak Ruins doorway room, 5, 6)</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>Check the tiles against the puzzle, or move one</t>
+          <t>Settled 2026-10-24: Landorus moved to the sand field</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
E10 part 25: Manaphy hatches from Backlot's Egg (a battle)
After the Mansion siege, Backlot's maid shows the player his deep blue
Egg in the office. It hatches, and the frightened Manaphy attacks
(Lv. 40). It waits in the office until caught. Renegade gives the Egg,
but Mythicals are battled, never given (decision 26).

Adds a placeholder overworld sprite for Manaphy.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GWchBEmvk4PBQrxv1zyRVz
</commit_message>
<xml_diff>
--- a/docs/StaticEncounters.xlsx
+++ b/docs/StaticEncounters.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J93"/>
+  <dimension ref="A1:J94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -620,6 +620,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4078,12 +4079,12 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Articuno</t>
-        </is>
-      </c>
-      <c r="C77" s="12" t="inlineStr">
-        <is>
-          <t>Renegade (not ported yet)</t>
+          <t>Manaphy</t>
+        </is>
+      </c>
+      <c r="C77" s="11" t="inlineStr">
+        <is>
+          <t>Renegade (ported)</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -4093,30 +4094,30 @@
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>Mt. Coronet summit portal</t>
+          <t>Pokémon Mansion, Mr. Backlot's office</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>to place</t>
+          <t>(18, 7)</t>
         </is>
       </c>
       <c r="G77" s="4" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>After the Distortion World (decision 33)</t>
-        </is>
-      </c>
-      <c r="I77" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+          <t>After the Mansion siege: Backlot's maid shows his Egg and it hatches</t>
+        </is>
+      </c>
+      <c r="I77" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
-          <t>Keep it off Cosmog's tile (35, 21)</t>
+          <t>A battle, not Renegade's Egg gift (decision 26)</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4127,7 @@
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Zapdos</t>
+          <t>Articuno</t>
         </is>
       </c>
       <c r="C78" s="12" t="inlineStr">
@@ -4141,7 +4142,7 @@
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>Valley Windworks, the island</t>
+          <t>Mt. Coronet summit portal</t>
         </is>
       </c>
       <c r="F78" s="4" t="inlineStr">
@@ -4157,14 +4158,14 @@
           <t>After the Distortion World (decision 33)</t>
         </is>
       </c>
-      <c r="I78" s="9" t="inlineStr">
-        <is>
-          <t>Clash</t>
+      <c r="I78" s="8" t="inlineStr">
+        <is>
+          <t>Check</t>
         </is>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
-          <t>Zekrom stands on this island until it moves to Route 215</t>
+          <t>Keep it off Cosmog's tile (35, 21)</t>
         </is>
       </c>
     </row>
@@ -4174,7 +4175,7 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Moltres</t>
+          <t>Zapdos</t>
         </is>
       </c>
       <c r="C79" s="12" t="inlineStr">
@@ -4189,7 +4190,7 @@
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>Victory Road, a small room</t>
+          <t>Valley Windworks, the island</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr">
@@ -4205,12 +4206,16 @@
           <t>After the Distortion World (decision 33)</t>
         </is>
       </c>
-      <c r="I79" s="7" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="J79" s="6" t="inlineStr"/>
+      <c r="I79" s="9" t="inlineStr">
+        <is>
+          <t>Clash</t>
+        </is>
+      </c>
+      <c r="J79" s="6" t="inlineStr">
+        <is>
+          <t>Zekrom stands on this island until it moves to Route 215</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="n">
@@ -4218,7 +4223,7 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Lugia</t>
+          <t>Moltres</t>
         </is>
       </c>
       <c r="C80" s="12" t="inlineStr">
@@ -4233,7 +4238,7 @@
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
-          <t>Route 220 island</t>
+          <t>Victory Road, a small room</t>
         </is>
       </c>
       <c r="F80" s="4" t="inlineStr">
@@ -4242,11 +4247,11 @@
         </is>
       </c>
       <c r="G80" s="4" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>After the Hall of Fame, Silver Wing</t>
+          <t>After the Distortion World (decision 33)</t>
         </is>
       </c>
       <c r="I80" s="7" t="inlineStr">
@@ -4262,7 +4267,7 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Ho-Oh</t>
+          <t>Lugia</t>
         </is>
       </c>
       <c r="C81" s="12" t="inlineStr">
@@ -4277,7 +4282,7 @@
       </c>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t>Lost Tower top floor (5F)</t>
+          <t>Route 220 island</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
@@ -4290,19 +4295,15 @@
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>After the Hall of Fame, Rainbow Wing</t>
-        </is>
-      </c>
-      <c r="I81" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="J81" s="6" t="inlineStr">
-        <is>
-          <t>Yveltal has moved out. Keep the portal off Totem Marowak's tile (3, 4)</t>
-        </is>
-      </c>
+          <t>After the Hall of Fame, Silver Wing</t>
+        </is>
+      </c>
+      <c r="I81" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J81" s="6" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n">
@@ -4310,7 +4311,7 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Celebi</t>
+          <t>Ho-Oh</t>
         </is>
       </c>
       <c r="C82" s="12" t="inlineStr">
@@ -4325,7 +4326,7 @@
       </c>
       <c r="E82" s="6" t="inlineStr">
         <is>
-          <t>Eterna Forest portals</t>
+          <t>Lost Tower top floor (5F)</t>
         </is>
       </c>
       <c r="F82" s="4" t="inlineStr">
@@ -4334,11 +4335,11 @@
         </is>
       </c>
       <c r="G82" s="4" t="n">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>Renegade's trigger</t>
+          <t>After the Hall of Fame, Rainbow Wing</t>
         </is>
       </c>
       <c r="I82" s="8" t="inlineStr">
@@ -4348,7 +4349,7 @@
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
-          <t>Keep the portals off Virizion (80, 10), Xerneas (70, 14) and Totem Vikavolt (22, 68)</t>
+          <t>Yveltal has moved out. Keep the portal off Totem Marowak's tile (3, 4)</t>
         </is>
       </c>
     </row>
@@ -4358,43 +4359,47 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Totem Gumshoos</t>
-        </is>
-      </c>
-      <c r="C83" s="13" t="inlineStr">
-        <is>
-          <t>Totem trial</t>
+          <t>Celebi</t>
+        </is>
+      </c>
+      <c r="C83" s="12" t="inlineStr">
+        <is>
+          <t>Renegade (not ported yet)</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Totem</t>
+          <t>Renegade</t>
         </is>
       </c>
       <c r="E83" s="6" t="inlineStr">
         <is>
-          <t>Route 205 South, flower bed</t>
+          <t>Eterna Forest portals</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>(197, 656)</t>
+          <t>to place</t>
         </is>
       </c>
       <c r="G83" s="4" t="n">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>After Roark</t>
-        </is>
-      </c>
-      <c r="I83" s="7" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="J83" s="6" t="inlineStr"/>
+          <t>Renegade's trigger</t>
+        </is>
+      </c>
+      <c r="I83" s="8" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="J83" s="6" t="inlineStr">
+        <is>
+          <t>Keep the portals off Virizion (80, 10), Xerneas (70, 14) and Totem Vikavolt (22, 68)</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="n">
@@ -4402,7 +4407,7 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Totem Ribombee</t>
+          <t>Totem Gumshoos</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
@@ -4417,32 +4422,28 @@
       </c>
       <c r="E84" s="6" t="inlineStr">
         <is>
-          <t>Floaroma Meadow</t>
+          <t>Route 205 South, flower bed</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>(18, 43)</t>
+          <t>(197, 656)</t>
         </is>
       </c>
       <c r="G84" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>After Mars (Valley Windworks)</t>
-        </is>
-      </c>
-      <c r="I84" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="J84" s="6" t="inlineStr">
-        <is>
-          <t>Tapu Bulu (24, 36) on the same map, post-game</t>
-        </is>
-      </c>
+          <t>After Roark</t>
+        </is>
+      </c>
+      <c r="I84" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J84" s="6" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
@@ -4450,7 +4451,7 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Totem Vikavolt</t>
+          <t>Totem Ribombee</t>
         </is>
       </c>
       <c r="C85" s="13" t="inlineStr">
@@ -4465,20 +4466,20 @@
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t>Eterna Forest, clearing</t>
+          <t>Floaroma Meadow</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>(22, 68)</t>
+          <t>(18, 43)</t>
         </is>
       </c>
       <c r="G85" s="4" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>After Mars</t>
+          <t>After Mars (Valley Windworks)</t>
         </is>
       </c>
       <c r="I85" s="8" t="inlineStr">
@@ -4488,7 +4489,7 @@
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
-          <t>Virizion and Xerneas post-game; far apart on the map</t>
+          <t>Tapu Bulu (24, 36) on the same map, post-game</t>
         </is>
       </c>
     </row>
@@ -4498,7 +4499,7 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Totem Mimikyu</t>
+          <t>Totem Vikavolt</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
@@ -4513,20 +4514,20 @@
       </c>
       <c r="E86" s="6" t="inlineStr">
         <is>
-          <t>Old Chateau dining area</t>
+          <t>Eterna Forest, clearing</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>(26, 10)</t>
+          <t>(22, 68)</t>
         </is>
       </c>
       <c r="G86" s="4" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>After Jupiter (Eterna)</t>
+          <t>After Mars</t>
         </is>
       </c>
       <c r="I86" s="8" t="inlineStr">
@@ -4536,7 +4537,7 @@
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
-          <t>Marshadow (21, 9) in the same room, post-game</t>
+          <t>Virizion and Xerneas post-game; far apart on the map</t>
         </is>
       </c>
     </row>
@@ -4546,7 +4547,7 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Totem Marowak (Alolan)</t>
+          <t>Totem Mimikyu</t>
         </is>
       </c>
       <c r="C87" s="13" t="inlineStr">
@@ -4561,20 +4562,20 @@
       </c>
       <c r="E87" s="6" t="inlineStr">
         <is>
-          <t>Lost Tower 5F, left of the stairs</t>
+          <t>Old Chateau dining area</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>(3, 4)</t>
+          <t>(26, 10)</t>
         </is>
       </c>
       <c r="G87" s="4" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>Relic Badge</t>
+          <t>After Jupiter (Eterna)</t>
         </is>
       </c>
       <c r="I87" s="8" t="inlineStr">
@@ -4584,7 +4585,7 @@
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
-          <t>Ho-Oh's portal goes on this floor (not ported yet). Yveltal moved out</t>
+          <t>Marshadow (21, 9) in the same room, post-game</t>
         </is>
       </c>
     </row>
@@ -4594,7 +4595,7 @@
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Totem Raticate (Alolan)</t>
+          <t>Totem Marowak (Alolan)</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
@@ -4609,28 +4610,32 @@
       </c>
       <c r="E88" s="6" t="inlineStr">
         <is>
-          <t>Galactic Warehouse, lower hall</t>
+          <t>Lost Tower 5F, left of the stairs</t>
         </is>
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>(13, 10)</t>
+          <t>(3, 4)</t>
         </is>
       </c>
       <c r="G88" s="4" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="H88" s="6" t="inlineStr">
         <is>
           <t>Relic Badge</t>
         </is>
       </c>
-      <c r="I88" s="7" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="J88" s="6" t="inlineStr"/>
+      <c r="I88" s="8" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="J88" s="6" t="inlineStr">
+        <is>
+          <t>Ho-Oh's portal goes on this floor (not ported yet). Yveltal moved out</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n">
@@ -4638,7 +4643,7 @@
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Totem Lurantis</t>
+          <t>Totem Raticate (Alolan)</t>
         </is>
       </c>
       <c r="C89" s="13" t="inlineStr">
@@ -4653,20 +4658,20 @@
       </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>Great Marsh Area 3</t>
+          <t>Galactic Warehouse, lower hall</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>(54, 84)</t>
+          <t>(13, 10)</t>
         </is>
       </c>
       <c r="G89" s="4" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>Cobble Badge (Safari Game)</t>
+          <t>Relic Badge</t>
         </is>
       </c>
       <c r="I89" s="7" t="inlineStr">
@@ -4682,7 +4687,7 @@
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Totem Araquanid</t>
+          <t>Totem Lurantis</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
@@ -4697,32 +4702,28 @@
       </c>
       <c r="E90" s="6" t="inlineStr">
         <is>
-          <t>Route 213, beach below the hotel</t>
+          <t>Great Marsh Area 3</t>
         </is>
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>(713, 826)</t>
+          <t>(54, 84)</t>
         </is>
       </c>
       <c r="G90" s="4" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>Fen Badge</t>
-        </is>
-      </c>
-      <c r="I90" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="J90" s="6" t="inlineStr">
-        <is>
-          <t>Suicune (689, 826) on the same route, 24 tiles west</t>
-        </is>
-      </c>
+          <t>Cobble Badge (Safari Game)</t>
+        </is>
+      </c>
+      <c r="I90" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J90" s="6" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="n">
@@ -4730,7 +4731,7 @@
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Totem Salazzle</t>
+          <t>Totem Araquanid</t>
         </is>
       </c>
       <c r="C91" s="13" t="inlineStr">
@@ -4745,20 +4746,20 @@
       </c>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t>Fuego Ironworks outside, north of the yard</t>
+          <t>Route 213, beach below the hotel</t>
         </is>
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>(181, 585)</t>
+          <t>(713, 826)</t>
         </is>
       </c>
       <c r="G91" s="4" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>After Cyrus (Celestic)</t>
+          <t>Fen Badge</t>
         </is>
       </c>
       <c r="I91" s="8" t="inlineStr">
@@ -4768,7 +4769,7 @@
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
-          <t>Chi-Yu (180, 593) and its stakes on the same map, post-game</t>
+          <t>Suicune (689, 826) on the same route, 24 tiles west</t>
         </is>
       </c>
     </row>
@@ -4778,7 +4779,7 @@
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Totem Kommo-o</t>
+          <t>Totem Salazzle</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
@@ -4793,28 +4794,32 @@
       </c>
       <c r="E92" s="6" t="inlineStr">
         <is>
-          <t>Mt. Coronet 6F</t>
+          <t>Fuego Ironworks outside, north of the yard</t>
         </is>
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>(5, 13)</t>
+          <t>(181, 585)</t>
         </is>
       </c>
       <c r="G92" s="4" t="n">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>After Saturn (Galactic HQ)</t>
-        </is>
-      </c>
-      <c r="I92" s="7" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="J92" s="6" t="inlineStr"/>
+          <t>After Cyrus (Celestic)</t>
+        </is>
+      </c>
+      <c r="I92" s="8" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="J92" s="6" t="inlineStr">
+        <is>
+          <t>Chi-Yu (180, 593) and its stakes on the same map, post-game</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="n">
@@ -4822,43 +4827,87 @@
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
+          <t>Totem Kommo-o</t>
+        </is>
+      </c>
+      <c r="C93" s="13" t="inlineStr">
+        <is>
+          <t>Totem trial</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>Totem</t>
+        </is>
+      </c>
+      <c r="E93" s="6" t="inlineStr">
+        <is>
+          <t>Mt. Coronet 6F</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>(5, 13)</t>
+        </is>
+      </c>
+      <c r="G93" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="H93" s="6" t="inlineStr">
+        <is>
+          <t>After Saturn (Galactic HQ)</t>
+        </is>
+      </c>
+      <c r="I93" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J93" s="6" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
           <t>Totem Togedemaru</t>
         </is>
       </c>
-      <c r="C93" s="13" t="inlineStr">
+      <c r="C94" s="13" t="inlineStr">
         <is>
           <t>Totem trial</t>
         </is>
       </c>
-      <c r="D93" s="4" t="inlineStr">
+      <c r="D94" s="4" t="inlineStr">
         <is>
           <t>Totem</t>
         </is>
       </c>
-      <c r="E93" s="6" t="inlineStr">
+      <c r="E94" s="6" t="inlineStr">
         <is>
           <t>Vista Lighthouse, top floor</t>
         </is>
       </c>
-      <c r="F93" s="4" t="inlineStr">
+      <c r="F94" s="4" t="inlineStr">
         <is>
           <t>(10, 7)</t>
         </is>
       </c>
-      <c r="G93" s="4" t="n">
+      <c r="G94" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="H93" s="6" t="inlineStr">
+      <c r="H94" s="6" t="inlineStr">
         <is>
           <t>After the Distortion World</t>
         </is>
       </c>
-      <c r="I93" s="8" t="inlineStr">
+      <c r="I94" s="8" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="J93" s="6" t="inlineStr">
+      <c r="J94" s="6" t="inlineStr">
         <is>
           <t>Victini (2, 7) on the same floor, post-game</t>
         </is>

</xml_diff>

<commit_message>
Move Volcanion to Stark Mountain room 2; overworld size classes; Regional Forms Park levels and signs
Volcanion leaves room 1 (Groudon's) for room 2's north-east dead end.
The legendaries' overworld placeholders follow the owner's size classes:
Eternatus extra large (128x64, on Giratina Origin's model), the owner's
large list at 64x64, everything else 32x32 until sorted
(docs/OverworldSpriteSizes.md). The Regional Forms Park gets levels
40-55, 60 for the rare forms and 70 for the Galarian birds, and a sign
at the way into each zone.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sispid5Qo8kvdYnx3crKZR
</commit_message>
<xml_diff>
--- a/docs/StaticEncounters.xlsx
+++ b/docs/StaticEncounters.xlsx
@@ -187,10 +187,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1553,12 +1553,12 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Stark Mountain room 1</t>
+          <t>Stark Mountain room 2, north-east dead-end tunnel</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>(34, 24)</t>
+          <t>(73, 15)</t>
         </is>
       </c>
       <c r="G23" s="4" t="n">
@@ -1569,14 +1569,14 @@
           <t>Kalos Chronicle open</t>
         </is>
       </c>
-      <c r="I23" s="9" t="inlineStr">
-        <is>
-          <t>Clash</t>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>Shares room 1 with Groudon (6, 6) and the first-visit Galactic scene. Move one</t>
+          <t>MOVED 2026-10-24 from room 1 (34, 24), which Groudon uses. Room 2 has trainers and Buck's escort, but the tunnel is a dead end</t>
         </is>
       </c>
     </row>
@@ -3833,14 +3833,14 @@
           <t>After the Hall of Fame (Steven's Orbs)</t>
         </is>
       </c>
-      <c r="I71" s="9" t="inlineStr">
-        <is>
-          <t>Clash</t>
+      <c r="I71" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>Shares room 1 with Volcanion (34, 24)</t>
+          <t>Volcanion moved to room 2 on 2026-10-24</t>
         </is>
       </c>
     </row>
@@ -4910,22 +4910,22 @@
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Stark Mountain room 1</t>
+          <t>Stark Mountain</t>
         </is>
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>Volcanion (34, 24); Groudon (6, 6); first-visit Galactic scene</t>
+          <t>Groudon (room 1, 6, 6); Volcanion (room 2, 73, 15); Heatran (room 3)</t>
         </is>
       </c>
       <c r="C2" s="16" t="inlineStr">
         <is>
-          <t>Clash</t>
+          <t>None</t>
         </is>
       </c>
       <c r="D2" s="15" t="inlineStr">
         <is>
-          <t>Move Volcanion or Groudon</t>
+          <t>Settled 2026-10-24: Volcanion moved to room 2</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
           <t>Jirachi (Room 7, 5, 3); Hoopa (Room 6 north-west dead end, 2, 3)</t>
         </is>
       </c>
-      <c r="C3" s="17" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -4962,7 +4962,7 @@
           <t>Giratina (its room); Eternatus (Victory Road B1F, 14, 19)</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -4984,7 +4984,7 @@
           <t>Landorus (782, 323, outside); Regidrago (Rock Peak Ruins doorway room, 5, 6)</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -5006,7 +5006,7 @@
           <t>Zekrom (236, 650); Zapdos portal (to place)</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
         <is>
           <t>Clash</t>
         </is>
@@ -5402,7 +5402,7 @@
           <t>Enamorus (912, 535); Pecharunt (898, 526); Shaymin tablet (908, 491)</t>
         </is>
       </c>
-      <c r="C24" s="17" t="inlineStr">
+      <c r="C24" s="16" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -5424,7 +5424,7 @@
           <t>Yveltal (813, 426); Gene (827, 438)</t>
         </is>
       </c>
-      <c r="C25" s="17" t="inlineStr">
+      <c r="C25" s="16" t="inlineStr">
         <is>
           <t>None</t>
         </is>

</xml_diff>

<commit_message>
E10 part 26: Snowpoint Temple story and HM08; Paradox rumours; Infinite Repel
Renegade's Snowpoint chapter (decision 29):
- Regigigas stirs under the temple. The town shakes, the townspeople talk
  about it, and the Gym guide blocks the Gym door while Candice is away.
- Two Ace Trainers (Renegade's 936/937) let only the strong into the temple,
  after a double battle.
- On B5F, Candice and Maylene put Regigigas back to sleep with the player,
  and Candice gives HM08. Regigigas itself also waits for the Champion now.
- The Route 217 hiker heals the party instead.

Decision 30: the museum dealers' all-given lines point to Sendoff Spring.
Decision 31: the home PC gives the Infinite Repel after the first Champion
win.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GWchBEmvk4PBQrxv1zyRVz
</commit_message>
<xml_diff>
--- a/docs/StaticEncounters.xlsx
+++ b/docs/StaticEncounters.xlsx
@@ -3275,7 +3275,7 @@
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>Regirock, Regice, Registeel in the party</t>
+          <t>After the Hall of Fame; Regirock, Regice, Registeel in the party</t>
         </is>
       </c>
       <c r="I59" s="7" t="inlineStr">
@@ -3283,7 +3283,11 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J59" s="6" t="inlineStr"/>
+      <c r="J59" s="6" t="inlineStr">
+        <is>
+          <t>Renegade's story scene (Candice, Maylene, HM08) stands beside it before the Gym (decision 29)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="n">

</xml_diff>

<commit_message>
E10 part 27: Articuno, Zapdos and Moltres where Renegade's portals stood
Decision 33: the birds no longer roam. Each is a Lv. 60 static from the
Distortion World on, until caught, like Raikou: Articuno on Mt. Coronet's
top snowfield (33, 20) beside Cosmog, Zapdos on the island north of
Valley Windworks (241, 644) beside the TM24 ball, Moltres in Victory
Road 2F's boulder room (20, 3), clear of the puzzle's tiles. Victory
Road 2F gets its own script archive. The Mt. Coronet and Valley
Windworks removals now check which species was battled.

Professor Oak gives the Up-Grade with a hint at the three places instead
of releasing roamers; his all-caught praise reads the Pokédex and waits
until after his first talk. Placeholder overworld sprites, docs and
CB-0101.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GWchBEmvk4PBQrxv1zyRVz
</commit_message>
<xml_diff>
--- a/docs/StaticEncounters.xlsx
+++ b/docs/StaticEncounters.xlsx
@@ -620,7 +620,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1092,12 +1091,12 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Clash</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>Zapdos's Renegade portal is on this island. Decision 34: Zekrom moves to Route 215 (tile to pick)</t>
+          <t>Zapdos stands on the small north island (241, 644), not this one (E10 part 27). Decision 34 (move to Route 215, tile to pick) still stands</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1816,7 @@
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Articuno's Renegade summit portal goes nearby: keep it off (35, 21)</t>
+          <t>Articuno (33, 20) stands two tiles away (E10 part 27)</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2296,7 @@
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>MOVED 2026-10-24 from Turnback Cave's Giratina room (8, 13). Shares the island with the TM59 ball (13, 18); Moltres's portal is in a 1F room</t>
+          <t>MOVED 2026-10-24 from Turnback Cave's Giratina room (8, 13). Shares the island with the TM59 ball (13, 18); Moltres stands on 2F (20, 3)</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2532,7 @@
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>Inside map; Zekrom/Zapdos are on the outside map</t>
+          <t>Inside map; Zekrom and Zapdos are on the outside map</t>
         </is>
       </c>
     </row>
@@ -4136,7 +4135,7 @@
       </c>
       <c r="C78" s="12" t="inlineStr">
         <is>
-          <t>Renegade (not ported yet)</t>
+          <t>Renegade (ported)</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -4146,12 +4145,12 @@
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>Mt. Coronet summit portal</t>
+          <t>Mt. Coronet outside north, top snowfield</t>
         </is>
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>to place</t>
+          <t>(33, 20)</t>
         </is>
       </c>
       <c r="G78" s="4" t="n">
@@ -4169,7 +4168,7 @@
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
-          <t>Keep it off Cosmog's tile (35, 21)</t>
+          <t>E10 part 27. Two tiles from Cosmog (35, 21), on its own hidden flag; Renegade's portal was at (35, 20)</t>
         </is>
       </c>
     </row>
@@ -4184,7 +4183,7 @@
       </c>
       <c r="C79" s="12" t="inlineStr">
         <is>
-          <t>Renegade (not ported yet)</t>
+          <t>Renegade (ported)</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -4194,12 +4193,12 @@
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>Valley Windworks, the island</t>
+          <t>Valley Windworks outside, the small island north of the building (Surf)</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>to place</t>
+          <t>(241, 644)</t>
         </is>
       </c>
       <c r="G79" s="4" t="n">
@@ -4212,12 +4211,12 @@
       </c>
       <c r="I79" s="9" t="inlineStr">
         <is>
-          <t>Clash</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
-          <t>Zekrom stands on this island until it moves to Route 215</t>
+          <t>E10 part 27. Beside the TM24 ball (242, 644), Renegade's portal tile; Zekrom (236, 650) is on the west island</t>
         </is>
       </c>
     </row>
@@ -4232,7 +4231,7 @@
       </c>
       <c r="C80" s="12" t="inlineStr">
         <is>
-          <t>Renegade (not ported yet)</t>
+          <t>Renegade (ported)</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -4242,12 +4241,12 @@
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
-          <t>Victory Road, a small room</t>
+          <t>Victory Road 2F, the small room past the Strength boulders</t>
         </is>
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>to place</t>
+          <t>(20, 3)</t>
         </is>
       </c>
       <c r="G80" s="4" t="n">
@@ -4260,10 +4259,14 @@
       </c>
       <c r="I80" s="7" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="J80" s="6" t="inlineStr"/>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="J80" s="6" t="inlineStr">
+        <is>
+          <t>E10 part 27. Off the tiles the boulder puzzle for TM79 needs (column 19 and (18, 3)); Renegade removed the boulders and used (18, 3)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n">
@@ -5056,17 +5059,17 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Zekrom (236, 650); Zapdos portal (to place)</t>
+          <t>Zekrom (236, 650, west island); Zapdos (241, 644, north island)</t>
         </is>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
-          <t>Clash</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>Move Zekrom to Route 215 (decision 34; tile to pick)</t>
+          <t>Different islands (E10 part 27). Decision 34 still moves Zekrom to Route 215 (tile to pick)</t>
         </is>
       </c>
     </row>
@@ -5078,7 +5081,7 @@
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>Kyurem (Iceberg doorway room, 7, 5); Regice's ruins; Cosmog (35, 21); Articuno portal (to place); Kyogre (B1F); Totem Kommo-o (6F)</t>
+          <t>Kyurem (Iceberg doorway room, 7, 5); Regice's ruins; Cosmog (35, 21); Articuno (33, 20); Kyogre (B1F); Totem Kommo-o (6F)</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
@@ -5088,7 +5091,7 @@
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>Kyurem works through a condition. Keep Articuno's portal off Cosmog's tile</t>
+          <t>Kyurem works through a condition. Articuno stands two tiles from Cosmog (E10 part 27)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
E10 part 28: Celebi, the GS Ball and the time portals in Eterna Forest
Renegade's Celebi event. The GS Ball (a new key item) waits in Celestic
Town's shrine; carried into Eterna Forest from the Eterna City side it
shakes, Celebi peeks out, and eight time portals open. Each holds the
memory of a battle with a Johto Gym Leader (Renegade's trainers
1029-1036). With all eight beaten, Celebi waits at (70, 58), Lv. 40,
until caught. VAR_SOVEREIGN_CELEBI_STATE takes over the unread
VAR_DUMMY_0x4083; the portals hide themselves off their trainers'
defeated flags.

Testing found that two CloseMessage in a row remove the message window
twice and hang the game; the portal script is fixed, and the new
tools/test/check_double_close.py finds no other Sovereign case.
Placeholder art: the GS Ball icon, the time portal and Celebi.
Docs and CB-0102.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GWchBEmvk4PBQrxv1zyRVz
</commit_message>
<xml_diff>
--- a/docs/StaticEncounters.xlsx
+++ b/docs/StaticEncounters.xlsx
@@ -812,7 +812,7 @@
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Shares the forest with Xerneas (70, 14) and Totem Vikavolt (22, 68); Celebi's Renegade portals still to place</t>
+          <t>Shares the forest with Xerneas (70, 14), Totem Vikavolt (22, 68) and Celebi (70, 58) with its portals (E10 part 28)</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>Same forest as Virizion (80, 10) and Totem Vikavolt; Celebi's portals still to place</t>
+          <t>Same forest as Virizion (80, 10), Totem Vikavolt and Celebi (70, 58)</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
       </c>
       <c r="C83" s="12" t="inlineStr">
         <is>
-          <t>Renegade (not ported yet)</t>
+          <t>Renegade (ported)</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -4381,12 +4381,12 @@
       </c>
       <c r="E83" s="6" t="inlineStr">
         <is>
-          <t>Eterna Forest portals</t>
+          <t>Eterna Forest, near the middle</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>to place</t>
+          <t>(70, 58)</t>
         </is>
       </c>
       <c r="G83" s="4" t="n">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>Renegade's trigger</t>
+          <t>GS Ball from Celestic Town, then the eight time portals</t>
         </is>
       </c>
       <c r="I83" s="8" t="inlineStr">
@@ -4404,7 +4404,7 @@
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
-          <t>Keep the portals off Virizion (80, 10), Xerneas (70, 14) and Totem Vikavolt (22, 68)</t>
+          <t>E10 part 28. Portals at (74, 32), (65, 34), (82, 46), (81, 72), (53, 60), (41, 58), (29, 64), (24, 68), all clear of Virizion, Xerneas and Totem Vikavolt</t>
         </is>
       </c>
     </row>
@@ -5103,7 +5103,7 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Virizion (80, 10); Xerneas (70, 14); Totem Vikavolt (22, 68); Celebi portals (to place)</t>
+          <t>Virizion (80, 10); Xerneas (70, 14); Totem Vikavolt (22, 68); Celebi (70, 58) and its eight time portals</t>
         </is>
       </c>
       <c r="C8" s="18" t="inlineStr">
@@ -5113,7 +5113,7 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>Place Celebi's portals clear of all three</t>
+          <t>Settled in E10 part 28: the portals keep Renegade's tiles, clear of all three (the one beside Totem Vikavolt moved to (24, 68))</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
E10 part 29: Lugia and Ho-Oh with Professor Oak's Clear Wings
Renegade's QUESTS: once Oak has praised the three birds, his two Clear
Wings become the Silver Wing (Articuno, Zapdos and Moltres in the
party) and the Rainbow Wing (Raikou, Entei and Suicune), new key items.
Carried after the Hall of Fame, they bring Lugia to Route 220's sandbar
island (190, 921) and Ho-Oh to Lost Tower 5F below the graves (7, 12),
Lv. 70, until caught. Route 220 gets its own script archive. Large
placeholder overworld sprites, docs and CB-0103.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GWchBEmvk4PBQrxv1zyRVz
</commit_message>
<xml_diff>
--- a/docs/StaticEncounters.xlsx
+++ b/docs/StaticEncounters.xlsx
@@ -1384,7 +1384,7 @@
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>MOVED 2026-10-24 from Lost Tower 5F (13, 14), which holds Totem Marowak and Ho-Oh's planned portal. Next to the Reaper Cloth ball (816, 426); Gene at (827, 438)</t>
+          <t>MOVED 2026-10-24 from Lost Tower 5F (13, 14), which holds Totem Marowak and Ho-Oh (7, 12). Next to the Reaper Cloth ball (816, 426); Gene at (827, 438)</t>
         </is>
       </c>
     </row>
@@ -4279,7 +4279,7 @@
       </c>
       <c r="C81" s="12" t="inlineStr">
         <is>
-          <t>Renegade (not ported yet)</t>
+          <t>Renegade (ported)</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -4289,12 +4289,12 @@
       </c>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t>Route 220 island</t>
+          <t>Route 220, the sandbar island at the bottom (Surf)</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>to place</t>
+          <t>(190, 921)</t>
         </is>
       </c>
       <c r="G81" s="4" t="n">
@@ -4310,7 +4310,11 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J81" s="6" t="inlineStr"/>
+      <c r="J81" s="6" t="inlineStr">
+        <is>
+          <t>E10 part 29. Oak gives the Silver Wing with Articuno, Zapdos and Moltres in the party</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n">
@@ -4323,7 +4327,7 @@
       </c>
       <c r="C82" s="12" t="inlineStr">
         <is>
-          <t>Renegade (not ported yet)</t>
+          <t>Renegade (ported)</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -4333,12 +4337,12 @@
       </c>
       <c r="E82" s="6" t="inlineStr">
         <is>
-          <t>Lost Tower top floor (5F)</t>
+          <t>Lost Tower 5F, below the old women's graves</t>
         </is>
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>to place</t>
+          <t>(7, 12)</t>
         </is>
       </c>
       <c r="G82" s="4" t="n">
@@ -4356,7 +4360,7 @@
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
-          <t>Yveltal has moved out. Keep the portal off Totem Marowak's tile (3, 4)</t>
+          <t>E10 part 29. Clear of Totem Marowak's tile (3, 4). Oak gives the Rainbow Wing with Raikou, Entei and Suicune in the party</t>
         </is>
       </c>
     </row>
@@ -4640,7 +4644,7 @@
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
-          <t>Ho-Oh's portal goes on this floor (not ported yet). Yveltal moved out</t>
+          <t>Ho-Oh stands on this floor at (7, 12), after the Hall of Fame (E10 part 29). Yveltal moved out</t>
         </is>
       </c>
     </row>
@@ -5125,7 +5129,7 @@
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>Totem Marowak (3, 4); Ho-Oh portal (to place)</t>
+          <t>Totem Marowak (3, 4); Ho-Oh (7, 12)</t>
         </is>
       </c>
       <c r="C9" s="18" t="inlineStr">
@@ -5135,7 +5139,7 @@
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>Settled for Yveltal (moved 2026-10-24). Keep Ho-Oh off (3, 4)</t>
+          <t>Settled for Yveltal (moved 2026-10-24). Ho-Oh stands at (7, 12), clear of Marowak (E10 part 29)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
E10 part 38: Renegade's Arceus (the Foreign Building elder's Plates and Azure Flute, no distribution)
- A new elder in Hearthome's Foreign Building (Renegade's lines) gives the Azure Flute once all sixteen Type
  Masters' Plates are in the bag. Renegade's Pokedex task is dropped (owner, decision 44).
- The Arceus distribution checks are gone from the flute's use check and common script, the Hall of Origin and
  the three Spear Pillar maps. Arceus stays Lv. 80.
- docs/StaticEncounters.xlsx gives Darkrai's and Arceus's new conditions; its generator is synced with the
  workbook again.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GWchBEmvk4PBQrxv1zyRVz
</commit_message>
<xml_diff>
--- a/docs/StaticEncounters.xlsx
+++ b/docs/StaticEncounters.xlsx
@@ -3366,11 +3366,11 @@
         </is>
       </c>
       <c r="G61" s="4" t="n">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>Member Card</t>
+          <t>Member Card (Route 217 woman, Lunar Wing)</t>
         </is>
       </c>
       <c r="I61" s="7" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>Azure Flute</t>
+          <t>Azure Flute (Foreign Building elder, 16 Plates)</t>
         </is>
       </c>
       <c r="I63" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Decision 34: Zekrom moves to Route 215; the placement review is closed
Zekrom now stands on Route 215's north-west loop by the big tree (590, 578),
with its unchanged trigger (the Dark Stone, at night). Valley Windworks
keeps Zapdos alone; its script entry is renumbered. The Archivist's hint
points to rainy Route 215.

Clash 8 (Kyurem's doorway, Articuno by Cosmog) is settled as working by
design, and every Check verdict in docs/StaticEncounters.xlsx is now None
with its reason, from the tile check or the timing.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GWchBEmvk4PBQrxv1zyRVz
</commit_message>
<xml_diff>
--- a/docs/StaticEncounters.xlsx
+++ b/docs/StaticEncounters.xlsx
@@ -51,17 +51,17 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -89,11 +89,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4A8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
@@ -110,6 +105,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F4B6B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4A8"/>
       </patternFill>
     </fill>
     <fill>
@@ -144,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -163,7 +163,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -172,31 +172,25 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -205,16 +199,16 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -600,7 +594,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sovereign Platinum: static encounters, including Totems (2026-10-24)</t>
+          <t>Sovereign Platinum: static encounters, including Totems (2026-10-25)</t>
         </is>
       </c>
     </row>
@@ -796,14 +790,14 @@
           <t>Unova Chronicle open</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Shares the forest with Xerneas (70, 14), Totem Vikavolt (22, 68) and Celebi (70, 58) with its portals (E10 part 28)</t>
+          <t>Tile check 2026-10-25: clear. Shares the forest with Xerneas (70, 14), Totem Vikavolt (22, 68) and Celebi (70, 58) with its portals (E10 part 28)</t>
         </is>
       </c>
     </row>
@@ -888,14 +882,14 @@
           <t>Unova Chronicle open</t>
         </is>
       </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Same floor as Totem Togedemaru (10, 7) and the Electric Master (4, 3). Fine once the Totem trial is done; both stand if the trial was skipped</t>
+          <t>Tile check 2026-10-25: clear. Same floor as Totem Togedemaru (10, 7) and the Electric Master (4, 3); reachable even while both stand</t>
         </is>
       </c>
     </row>
@@ -936,14 +930,14 @@
           <t>Composer hears Sing</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>Uses the no-contest stage map; check it never shows during a contest</t>
+          <t>Contests use their own stage map (CONTEST_HALL_STAGE_ONGOING_CONTEST), so it never shows during one. Tile check 2026-10-25: clear.</t>
         </is>
       </c>
     </row>
@@ -1064,12 +1058,12 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Valley Windworks outside, the island (moving)</t>
+          <t>Route 215, the north-west loop by the big tree</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>(236, 650)</t>
+          <t>(590, 578)</t>
         </is>
       </c>
       <c r="G13" s="4" t="n">
@@ -1080,14 +1074,14 @@
           <t>Dark Stone in the bag, night</t>
         </is>
       </c>
-      <c r="I13" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>Zapdos stands on the small north island (241, 644), not this one (E10 part 27). Decision 34 (move to Route 215, tile to pick) still stands</t>
+          <t>MOVED 2026-10-25 from Valley Windworks' island (236, 650), decision 34. Tile check: clear</t>
         </is>
       </c>
     </row>
@@ -1128,14 +1122,14 @@
           <t>Reshiram and Zekrom caught; no Relicanth+Wailord pair</t>
         </is>
       </c>
-      <c r="I14" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>The Relicanth/Wailord pair swaps this room to Regice's chamber. Works through a condition, but fragile</t>
+          <t>The Relicanth/Wailord pair sends the doorway to Regice's chamber; without the pair it leads here. Works as designed (checked 2026-10-25)</t>
         </is>
       </c>
     </row>
@@ -1320,14 +1314,14 @@
           <t>Kalos Chronicle open</t>
         </is>
       </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>Same forest as Virizion (80, 10), Totem Vikavolt and Celebi (70, 58)</t>
+          <t>Tile check 2026-10-25: clear. Same forest as Virizion (80, 10), Totem Vikavolt and Celebi (70, 58)</t>
         </is>
       </c>
     </row>
@@ -1464,14 +1458,14 @@
           <t>Carbink in the party</t>
         </is>
       </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>Meltan (5, 20) and Melmetal (5, 24) within 4 tiles; check none blocks the path</t>
+          <t>Tile check 2026-10-25: clear. Meltan (5, 20) and Melmetal (5, 24) within 4 tiles; none blocks the path</t>
         </is>
       </c>
     </row>
@@ -1656,14 +1650,14 @@
           <t>Alola Chronicle open</t>
         </is>
       </c>
-      <c r="I25" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>Three tiles from Cresselia's / the Lati rock's tile (16, 15). Sequenced, but crowded</t>
+          <t>Tile check 2026-10-25: clear. Three tiles from Cresselia's / the Lati rock's tile (16, 15), which are sequenced</t>
         </is>
       </c>
     </row>
@@ -1704,14 +1698,14 @@
           <t>Alola Chronicle open</t>
         </is>
       </c>
-      <c r="I26" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>Totem Ribombee (18, 43) on the same map; the Grass Master at (47, 41)</t>
+          <t>Tile check 2026-10-25: clear. Totem Ribombee (18, 43) on the same map; the Grass Master at (47, 41)</t>
         </is>
       </c>
     </row>
@@ -1752,14 +1746,14 @@
           <t>Alola Chronicle open</t>
         </is>
       </c>
-      <c r="I27" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>Wyver (Renegade NPC) stands at (717, 346), the next tile. Check it doesn't block the encounter</t>
+          <t>Tile check 2026-10-25: clear. Wyver (Renegade NPC) stands at (717, 346), diagonal to it; it can be reached even with Wyver in the way</t>
         </is>
       </c>
     </row>
@@ -1800,14 +1794,14 @@
           <t>Alola Chronicle open</t>
         </is>
       </c>
-      <c r="I28" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Articuno (33, 20) stands two tiles away (E10 part 27)</t>
+          <t>Tile check 2026-10-25: clear. Articuno (33, 20) stands two tiles away (E10 part 27)</t>
         </is>
       </c>
     </row>
@@ -1848,14 +1842,14 @@
           <t>Solgaleo or Lunala caught</t>
         </is>
       </c>
-      <c r="I29" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>Mira's Renegade quest is in Wayward Cave</t>
+          <t>Tile check 2026-10-25: clear. Through the hidden entrance, past Mira's gate (her Renegade quest)</t>
         </is>
       </c>
     </row>
@@ -1944,14 +1938,14 @@
           <t>Alola Chronicle open</t>
         </is>
       </c>
-      <c r="I31" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>Beside Volkner; check it doesn't block his rematch or the exit</t>
+          <t>Tile check 2026-10-25: clear. Beside Volkner; it blocks neither his rematch nor the exit</t>
         </is>
       </c>
     </row>
@@ -1992,14 +1986,14 @@
           <t>Alola Chronicle open</t>
         </is>
       </c>
-      <c r="I32" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>Totem Mimikyu (26, 10) in the same room. Fine once the trial is done; both stand if it was skipped</t>
+          <t>Tile check 2026-10-25: clear. Totem Mimikyu (26, 10) in the same room; reachable even while it stands</t>
         </is>
       </c>
     </row>
@@ -2088,14 +2082,14 @@
           <t>Alola Chronicle open</t>
         </is>
       </c>
-      <c r="I34" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>See Diancie</t>
+          <t>Tile check 2026-10-25: clear. See Diancie</t>
         </is>
       </c>
     </row>
@@ -2136,14 +2130,14 @@
           <t>Meltan caught</t>
         </is>
       </c>
-      <c r="I35" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>See Diancie</t>
+          <t>Tile check 2026-10-25: clear. See Diancie</t>
         </is>
       </c>
     </row>
@@ -2328,14 +2322,14 @@
           <t>Galar Chronicle open</t>
         </is>
       </c>
-      <c r="I39" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>Check it isn't on the path to the ruins or the elder</t>
+          <t>Tile check 2026-10-25: clear. Off the paths to the ruins and the elder</t>
         </is>
       </c>
     </row>
@@ -2424,14 +2418,14 @@
           <t>Galar Chronicle open</t>
         </is>
       </c>
-      <c r="I41" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t>Inside the Gym; check it doesn't block the punching-bag puzzle</t>
+          <t>Tile check 2026-10-25: clear. Off every punching-bag track (the Gym's track table in src/overlay008/gym_features.c)</t>
         </is>
       </c>
     </row>
@@ -2748,14 +2742,14 @@
           <t>Stakes 7 and 8 pulled</t>
         </is>
       </c>
-      <c r="I48" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I48" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>Totem Salazzle (181, 585) on the same map, 8 tiles north</t>
+          <t>Tile check 2026-10-25: clear. Totem Salazzle (181, 585) on the same map, 8 tiles north</t>
         </is>
       </c>
     </row>
@@ -2940,14 +2934,14 @@
           <t>All ten ancient Paradox Pokémon traded</t>
         </is>
       </c>
-      <c r="I52" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I52" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>Miraidon (27, 37) and Terapagos (30, 34) within 3 tiles; check Cynthia's scene tiles</t>
+          <t>Cynthia's Sendoff Spring scene is before the Hall of Fame, and the Paldea Chronicle opens after it, so they never meet. Tile check 2026-10-25: clear.</t>
         </is>
       </c>
     </row>
@@ -2988,9 +2982,9 @@
           <t>All ten future Paradox Pokémon traded</t>
         </is>
       </c>
-      <c r="I53" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I53" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J53" s="6" t="inlineStr">
@@ -3036,9 +3030,9 @@
           <t>Koraidon and Miraidon caught</t>
         </is>
       </c>
-      <c r="I54" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I54" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J54" s="6" t="inlineStr">
@@ -3056,7 +3050,7 @@
           <t>Uxie / Mesprit / Azelf</t>
         </is>
       </c>
-      <c r="C55" s="9" t="inlineStr">
+      <c r="C55" s="8" t="inlineStr">
         <is>
           <t>Vanilla</t>
         </is>
@@ -3100,7 +3094,7 @@
           <t>Dialga / Palkia</t>
         </is>
       </c>
-      <c r="C56" s="9" t="inlineStr">
+      <c r="C56" s="8" t="inlineStr">
         <is>
           <t>Vanilla</t>
         </is>
@@ -3144,7 +3138,7 @@
           <t>Giratina</t>
         </is>
       </c>
-      <c r="C57" s="9" t="inlineStr">
+      <c r="C57" s="8" t="inlineStr">
         <is>
           <t>Vanilla</t>
         </is>
@@ -3192,7 +3186,7 @@
           <t>Heatran</t>
         </is>
       </c>
-      <c r="C58" s="9" t="inlineStr">
+      <c r="C58" s="8" t="inlineStr">
         <is>
           <t>Vanilla</t>
         </is>
@@ -3240,7 +3234,7 @@
           <t>Regigigas</t>
         </is>
       </c>
-      <c r="C59" s="9" t="inlineStr">
+      <c r="C59" s="8" t="inlineStr">
         <is>
           <t>Vanilla</t>
         </is>
@@ -3288,7 +3282,7 @@
           <t>Cresselia</t>
         </is>
       </c>
-      <c r="C60" s="9" t="inlineStr">
+      <c r="C60" s="8" t="inlineStr">
         <is>
           <t>Vanilla</t>
         </is>
@@ -3316,14 +3310,14 @@
           <t>After the Lunar Wing quest</t>
         </is>
       </c>
-      <c r="I60" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I60" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
-          <t>Tapu Lele (13, 12) three tiles away; Latias/Latios take the same tile later</t>
+          <t>Tapu Lele (13, 12) three tiles away; Latias/Latios take the same tile only after Cresselia (sequenced). Tile check 2026-10-25: clear.</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3330,7 @@
           <t>Darkrai</t>
         </is>
       </c>
-      <c r="C61" s="9" t="inlineStr">
+      <c r="C61" s="8" t="inlineStr">
         <is>
           <t>Vanilla</t>
         </is>
@@ -3380,7 +3374,7 @@
           <t>Shaymin</t>
         </is>
       </c>
-      <c r="C62" s="9" t="inlineStr">
+      <c r="C62" s="8" t="inlineStr">
         <is>
           <t>Vanilla</t>
         </is>
@@ -3428,7 +3422,7 @@
           <t>Arceus</t>
         </is>
       </c>
-      <c r="C63" s="9" t="inlineStr">
+      <c r="C63" s="8" t="inlineStr">
         <is>
           <t>Vanilla</t>
         </is>
@@ -3472,7 +3466,7 @@
           <t>Rotom</t>
         </is>
       </c>
-      <c r="C64" s="9" t="inlineStr">
+      <c r="C64" s="8" t="inlineStr">
         <is>
           <t>Vanilla</t>
         </is>
@@ -3520,7 +3514,7 @@
           <t>Raikou</t>
         </is>
       </c>
-      <c r="C65" s="10" t="inlineStr">
+      <c r="C65" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -3564,7 +3558,7 @@
           <t>Entei</t>
         </is>
       </c>
-      <c r="C66" s="10" t="inlineStr">
+      <c r="C66" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -3612,7 +3606,7 @@
           <t>Suicune</t>
         </is>
       </c>
-      <c r="C67" s="10" t="inlineStr">
+      <c r="C67" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -3640,14 +3634,14 @@
           <t>After the Distortion World</t>
         </is>
       </c>
-      <c r="I67" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I67" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>Totem Araquanid (713, 826) on the same route, 24 tiles east</t>
+          <t>Tile check 2026-10-25: clear. Totem Araquanid (713, 826) on the same route, 24 tiles east</t>
         </is>
       </c>
     </row>
@@ -3660,7 +3654,7 @@
           <t>Regirock / Regice / Registeel</t>
         </is>
       </c>
-      <c r="C68" s="10" t="inlineStr">
+      <c r="C68" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -3688,14 +3682,14 @@
           <t>Relicanth and Wailord in the party</t>
         </is>
       </c>
-      <c r="I68" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I68" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>Iceberg: Kyurem's doorway room. Rock Peak is settled (Landorus moved)</t>
+          <t>Iceberg: the pair sends Mt. Coronet's doorway here instead of Kyurem's room (works as designed). Rock Peak is settled (Landorus moved)</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3702,7 @@
           <t>Latias / Latios</t>
         </is>
       </c>
-      <c r="C69" s="10" t="inlineStr">
+      <c r="C69" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -3756,7 +3750,7 @@
           <t>Kyogre</t>
         </is>
       </c>
-      <c r="C70" s="10" t="inlineStr">
+      <c r="C70" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -3800,7 +3794,7 @@
           <t>Groudon</t>
         </is>
       </c>
-      <c r="C71" s="10" t="inlineStr">
+      <c r="C71" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -3848,7 +3842,7 @@
           <t>Rayquaza</t>
         </is>
       </c>
-      <c r="C72" s="10" t="inlineStr">
+      <c r="C72" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -3896,7 +3890,7 @@
           <t>Mewtwo</t>
         </is>
       </c>
-      <c r="C73" s="10" t="inlineStr">
+      <c r="C73" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -3940,7 +3934,7 @@
           <t>Jirachi</t>
         </is>
       </c>
-      <c r="C74" s="10" t="inlineStr">
+      <c r="C74" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -3988,7 +3982,7 @@
           <t>Deoxys</t>
         </is>
       </c>
-      <c r="C75" s="10" t="inlineStr">
+      <c r="C75" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -4032,7 +4026,7 @@
           <t>Mew</t>
         </is>
       </c>
-      <c r="C76" s="10" t="inlineStr">
+      <c r="C76" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -4076,7 +4070,7 @@
           <t>Manaphy</t>
         </is>
       </c>
-      <c r="C77" s="10" t="inlineStr">
+      <c r="C77" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -4124,7 +4118,7 @@
           <t>Articuno</t>
         </is>
       </c>
-      <c r="C78" s="10" t="inlineStr">
+      <c r="C78" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -4152,14 +4146,14 @@
           <t>After the Distortion World (decision 33)</t>
         </is>
       </c>
-      <c r="I78" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I78" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
-          <t>E10 part 27. Two tiles from Cosmog (35, 21), on its own hidden flag; Renegade's portal was at (35, 20)</t>
+          <t>Tile check 2026-10-25: clear. E10 part 27. Two tiles from Cosmog (35, 21), on its own hidden flag; Renegade's portal was at (35, 20)</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4166,7 @@
           <t>Zapdos</t>
         </is>
       </c>
-      <c r="C79" s="10" t="inlineStr">
+      <c r="C79" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -4200,14 +4194,14 @@
           <t>After the Distortion World (decision 33)</t>
         </is>
       </c>
-      <c r="I79" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I79" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
-          <t>E10 part 27. Beside the TM24 ball (242, 644), Renegade's portal tile; Zekrom (236, 650) is on the west island</t>
+          <t>E10 part 27. Beside the TM24 ball (242, 644), Renegade's portal tile. Zekrom moved to Route 215 (2026-10-25), so the islands are Zapdos's alone. Tile check: clear</t>
         </is>
       </c>
     </row>
@@ -4220,7 +4214,7 @@
           <t>Moltres</t>
         </is>
       </c>
-      <c r="C80" s="10" t="inlineStr">
+      <c r="C80" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -4248,14 +4242,14 @@
           <t>After the Distortion World (decision 33)</t>
         </is>
       </c>
-      <c r="I80" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I80" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
-          <t>E10 part 27. Off the tiles the boulder puzzle for TM79 needs (column 19 and (18, 3)); Renegade removed the boulders and used (18, 3)</t>
+          <t>Tile check 2026-10-25: clear. E10 part 27. Off the tiles the boulder puzzle for TM79 needs (column 19 and (18, 3))</t>
         </is>
       </c>
     </row>
@@ -4268,7 +4262,7 @@
           <t>Lugia</t>
         </is>
       </c>
-      <c r="C81" s="10" t="inlineStr">
+      <c r="C81" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -4316,7 +4310,7 @@
           <t>Ho-Oh</t>
         </is>
       </c>
-      <c r="C82" s="10" t="inlineStr">
+      <c r="C82" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -4344,14 +4338,14 @@
           <t>After the Hall of Fame, Rainbow Wing</t>
         </is>
       </c>
-      <c r="I82" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I82" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
-          <t>E10 part 29. Clear of Totem Marowak's tile (3, 4). Oak gives the Rainbow Wing with Raikou, Entei and Suicune in the party</t>
+          <t>Tile check 2026-10-25: clear. E10 part 29. Clear of Totem Marowak's tile (3, 4). Oak gives the Rainbow Wing with Raikou, Entei and Suicune in the party</t>
         </is>
       </c>
     </row>
@@ -4364,7 +4358,7 @@
           <t>Celebi</t>
         </is>
       </c>
-      <c r="C83" s="10" t="inlineStr">
+      <c r="C83" s="9" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
@@ -4392,14 +4386,14 @@
           <t>GS Ball from Celestic Town, then the eight time portals</t>
         </is>
       </c>
-      <c r="I83" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I83" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
-          <t>E10 part 28. Portals at (74, 32), (65, 34), (82, 46), (81, 72), (53, 60), (41, 58), (29, 64), (24, 68), all clear of Virizion, Xerneas and Totem Vikavolt</t>
+          <t>Tile check 2026-10-25: clear. E10 part 28. Its eight portals are clear of Virizion, Xerneas and Totem Vikavolt</t>
         </is>
       </c>
     </row>
@@ -4412,7 +4406,7 @@
           <t>Totem Gumshoos</t>
         </is>
       </c>
-      <c r="C84" s="11" t="inlineStr">
+      <c r="C84" s="10" t="inlineStr">
         <is>
           <t>Totem trial</t>
         </is>
@@ -4456,7 +4450,7 @@
           <t>Totem Ribombee</t>
         </is>
       </c>
-      <c r="C85" s="11" t="inlineStr">
+      <c r="C85" s="10" t="inlineStr">
         <is>
           <t>Totem trial</t>
         </is>
@@ -4484,14 +4478,14 @@
           <t>After Mars (Valley Windworks)</t>
         </is>
       </c>
-      <c r="I85" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I85" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
-          <t>Tapu Bulu (24, 36) on the same map, post-game</t>
+          <t>Tile check 2026-10-25: clear. Tapu Bulu (24, 36) on the same map, post-game</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4498,7 @@
           <t>Totem Vikavolt</t>
         </is>
       </c>
-      <c r="C86" s="11" t="inlineStr">
+      <c r="C86" s="10" t="inlineStr">
         <is>
           <t>Totem trial</t>
         </is>
@@ -4532,14 +4526,14 @@
           <t>After Mars</t>
         </is>
       </c>
-      <c r="I86" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I86" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
-          <t>Virizion and Xerneas post-game; far apart on the map</t>
+          <t>Tile check 2026-10-25: clear. Virizion and Xerneas post-game; far apart on the map</t>
         </is>
       </c>
     </row>
@@ -4552,7 +4546,7 @@
           <t>Totem Mimikyu</t>
         </is>
       </c>
-      <c r="C87" s="11" t="inlineStr">
+      <c r="C87" s="10" t="inlineStr">
         <is>
           <t>Totem trial</t>
         </is>
@@ -4580,14 +4574,14 @@
           <t>After Jupiter (Eterna)</t>
         </is>
       </c>
-      <c r="I87" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I87" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
-          <t>Marshadow (21, 9) in the same room, post-game</t>
+          <t>Tile check 2026-10-25: clear. Marshadow (21, 9) in the same room, post-game</t>
         </is>
       </c>
     </row>
@@ -4600,7 +4594,7 @@
           <t>Totem Marowak (Alolan)</t>
         </is>
       </c>
-      <c r="C88" s="11" t="inlineStr">
+      <c r="C88" s="10" t="inlineStr">
         <is>
           <t>Totem trial</t>
         </is>
@@ -4628,14 +4622,14 @@
           <t>Relic Badge</t>
         </is>
       </c>
-      <c r="I88" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I88" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
-          <t>Ho-Oh stands on this floor at (7, 12), after the Hall of Fame (E10 part 29). Yveltal moved out</t>
+          <t>Tile check 2026-10-25: clear. Ho-Oh stands on this floor at (7, 12), after the Hall of Fame (E10 part 29). Yveltal moved out</t>
         </is>
       </c>
     </row>
@@ -4648,7 +4642,7 @@
           <t>Totem Raticate (Alolan)</t>
         </is>
       </c>
-      <c r="C89" s="11" t="inlineStr">
+      <c r="C89" s="10" t="inlineStr">
         <is>
           <t>Totem trial</t>
         </is>
@@ -4692,7 +4686,7 @@
           <t>Totem Lurantis</t>
         </is>
       </c>
-      <c r="C90" s="11" t="inlineStr">
+      <c r="C90" s="10" t="inlineStr">
         <is>
           <t>Totem trial</t>
         </is>
@@ -4736,7 +4730,7 @@
           <t>Totem Araquanid</t>
         </is>
       </c>
-      <c r="C91" s="11" t="inlineStr">
+      <c r="C91" s="10" t="inlineStr">
         <is>
           <t>Totem trial</t>
         </is>
@@ -4764,14 +4758,14 @@
           <t>Fen Badge</t>
         </is>
       </c>
-      <c r="I91" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I91" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
-          <t>Suicune (689, 826) on the same route, 24 tiles west</t>
+          <t>Tile check 2026-10-25: clear. Suicune (689, 826) on the same route, 24 tiles west</t>
         </is>
       </c>
     </row>
@@ -4784,7 +4778,7 @@
           <t>Totem Salazzle</t>
         </is>
       </c>
-      <c r="C92" s="11" t="inlineStr">
+      <c r="C92" s="10" t="inlineStr">
         <is>
           <t>Totem trial</t>
         </is>
@@ -4812,14 +4806,14 @@
           <t>After Cyrus (Celestic)</t>
         </is>
       </c>
-      <c r="I92" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I92" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
-          <t>Chi-Yu (180, 593) and its stakes on the same map, post-game</t>
+          <t>Tile check 2026-10-25: clear. Chi-Yu (180, 593) and its stakes on the same map, post-game</t>
         </is>
       </c>
     </row>
@@ -4832,7 +4826,7 @@
           <t>Totem Kommo-o</t>
         </is>
       </c>
-      <c r="C93" s="11" t="inlineStr">
+      <c r="C93" s="10" t="inlineStr">
         <is>
           <t>Totem trial</t>
         </is>
@@ -4876,7 +4870,7 @@
           <t>Totem Togedemaru</t>
         </is>
       </c>
-      <c r="C94" s="11" t="inlineStr">
+      <c r="C94" s="10" t="inlineStr">
         <is>
           <t>Totem trial</t>
         </is>
@@ -4904,14 +4898,14 @@
           <t>After the Distortion World</t>
         </is>
       </c>
-      <c r="I94" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="I94" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
-          <t>Victini (2, 7) on the same floor, post-game</t>
+          <t>Tile check 2026-10-25: clear. Victini (2, 7) on the same floor, post-game</t>
         </is>
       </c>
     </row>
@@ -4937,550 +4931,550 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Map</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Encounters there</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Conflict</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>What to do</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Stark Mountain</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>Groudon (room 1, 6, 6); Volcanion (room 2, 73, 15); Heatran (room 3)</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="D2" s="13" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>Settled 2026-10-24: Volcanion moved to room 2</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Solaceon Ruins</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Jirachi (Room 7, 5, 3); Hoopa (Room 6 north-west dead end, 2, 3)</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>Settled 2026-10-24: Hoopa moved to Room 6</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Turnback Cave / Victory Road B1F</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Giratina (its room); Eternatus (Victory Road B1F, 14, 19)</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Settled 2026-10-24: Eternatus moved to Victory Road B1F</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Route 228</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Landorus (782, 323, outside); Regidrago (Rock Peak Ruins doorway room, 5, 6)</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Settled 2026-10-24: Landorus moved to the sand field</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Valley Windworks outside</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Zekrom (236, 650, west island); Zapdos (241, 644, north island)</t>
-        </is>
-      </c>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Different islands (E10 part 27). Decision 34 still moves Zekrom to Route 215 (tile to pick)</t>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Zapdos (241, 644, north island); Regieleki (building)</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Settled 2026-10-25: Zekrom moved to Route 215 (decision 34)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Mt. Coronet</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Kyurem (Iceberg doorway room, 7, 5); Regice's ruins; Cosmog (35, 21); Articuno (33, 20); Kyogre (B1F); Totem Kommo-o (6F)</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>Kyurem works through a condition. Articuno stands two tiles from Cosmog (E10 part 27)</t>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Kyurem works by design: the Relicanth/Wailord pair swaps the doorway to Regice's chamber. Articuno stands two tiles from Cosmog. Tile check 2026-10-25: clear</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Eterna Forest</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Virizion (80, 10); Xerneas (70, 14); Totem Vikavolt (22, 68); Celebi (70, 58) and its eight time portals</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D8" s="13" t="inlineStr">
-        <is>
-          <t>Settled in E10 part 28: the portals keep Renegade's tiles, clear of all three (the one beside Totem Vikavolt moved to (24, 68))</t>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Tile check 2026-10-25: clear. Settled in E10 part 28: the portals keep Renegade's tiles, clear of all three (the one beside Totem Vikavolt moved to (24, 68))</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Lost Tower 5F</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Totem Marowak (3, 4); Ho-Oh (7, 12)</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Settled for Yveltal (moved 2026-10-24). Ho-Oh stands at (7, 12), clear of Marowak (E10 part 29)</t>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Tile check 2026-10-25: clear. Settled for Yveltal (moved 2026-10-24). Ho-Oh stands at (7, 12), clear of Marowak (E10 part 29)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Old Chateau dining area</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Totem Mimikyu (26, 10); Marshadow (21, 9)</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>Both stand only if the Totem trial was skipped. Different eras of play</t>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Tile check 2026-10-25: clear. Both stand only if the Totem trial was skipped. Different eras of play</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Vista Lighthouse top floor</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Totem Togedemaru (10, 7); Victini (2, 7); Electric Master (4, 3)</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>As above</t>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Tile check 2026-10-25: clear. As above</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Fuego Ironworks outside</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Totem Salazzle (181, 585); Chi-Yu (180, 593) and stakes 7–8</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>As above</t>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Tile check 2026-10-25: clear. As above</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Floaroma Meadow</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Totem Ribombee (18, 43); Tapu Bulu (24, 36)</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>As above</t>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Tile check 2026-10-25: clear. As above</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Route 213</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>Totem Araquanid (713, 826); Suicune (689, 826)</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>24 tiles apart; fine</t>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Tile check 2026-10-25: clear. 24 tiles apart; fine</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Route 226</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Tapu Fini (716, 345); Wyver (717, 346)</t>
         </is>
       </c>
-      <c r="C15" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>Adjacent tiles; check the encounter can be reached</t>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Tile check 2026-10-25: clear. Adjacent tiles; check the encounter can be reached</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Oreburgh Mine B2F</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Diancie (2, 22); Meltan (5, 20); Melmetal (5, 24)</t>
         </is>
       </c>
-      <c r="C16" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D16" s="13" t="inlineStr">
-        <is>
-          <t>Sequenced or conditional; check they don't block the path</t>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Tile check 2026-10-25: clear. Sequenced or conditional; check they don't block the path</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Fullmoon Island forest</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>Tapu Lele (13, 12); Cresselia then Latias/Latios (16, 15)</t>
         </is>
       </c>
-      <c r="C17" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>Sequenced; crowded but fine</t>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Tile check 2026-10-25: clear. Sequenced; crowded but fine</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>Sendoff Spring</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>Koraidon (29, 36); Miraidon (27, 37); Terapagos (30, 34)</t>
         </is>
       </c>
-      <c r="C18" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
-        <is>
-          <t>Check Cynthia's scene tiles</t>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Tile check 2026-10-25: clear. Check Cynthia's scene tiles</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Wayward Cave</t>
         </is>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>Zygarde (B1F 12, 4); Necrozma (1F 70, 9); Mira's quest</t>
         </is>
       </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="inlineStr">
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
         <is>
           <t>Checked 2026-10-25: Mira waits on 1F at the hidden entrance, Zygarde is on B1F</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>Sunyshore Gym, Volkner's room</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>Magearna (11, 13); Volkner</t>
         </is>
       </c>
-      <c r="C20" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D20" s="13" t="inlineStr">
-        <is>
-          <t>Check the rematch and exit</t>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Tile check 2026-10-25: clear. Check the rematch and exit</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>Veilstone Gym</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>Kubfu (13, 17); the Gym puzzle</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>Check the puzzle</t>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Tile check 2026-10-25: clear. Check the puzzle</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>Celestic Town</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>Calyrex (461, 527); the elder, the ruins path</t>
         </is>
       </c>
-      <c r="C22" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
-        <is>
-          <t>Check the ruins path</t>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Tile check 2026-10-25: clear. Check the ruins path</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>Contest Hall stage</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>Meloetta (27, 8)</t>
         </is>
       </c>
-      <c r="C23" s="15" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>Check it never shows during a contest</t>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Tile check 2026-10-25: clear. Check it never shows during a contest</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>Route 224</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>Enamorus (912, 535); Pecharunt (898, 526); Shaymin tablet (908, 491)</t>
         </is>
       </c>
-      <c r="C24" s="14" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>Settled 2026-10-24: Enamorus moved off the tablet</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>Route 229</t>
         </is>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>Yveltal (813, 426); Gene (827, 438)</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="D25" s="13" t="inlineStr">
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>Yveltal's new spot (2026-10-24)</t>
         </is>
@@ -5505,132 +5499,132 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Conflict</t>
         </is>
       </c>
-      <c r="B1" s="17" t="inlineStr"/>
+      <c r="B1" s="15" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Clash</t>
         </is>
       </c>
-      <c r="B2" s="17" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>Two encounters (or an encounter and a story scene) share a small room or tile and can stand at once. Must be settled.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Shares a map with another encounter, NPC or puzzle. Verify the tiles or timing in game.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Nothing found on the map.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr"/>
-      <c r="B5" s="17" t="inlineStr"/>
+      <c r="A5" s="14" t="inlineStr"/>
+      <c r="B5" s="15" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr"/>
+      <c r="B6" s="15" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Chronicle</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>Post-game Chronicles from the Legend Archivist (Canalave Library 2F).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Vanilla</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>Platinum's own legendaries.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Renegade (ported)</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Renegade Platinum's events already ported (E10).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>Renegade (not ported yet)</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Renegade's events still to port.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>Totem trial</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>Story Totem trials (data/totem_trials.yaml). Each hides once its trial is done.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr"/>
-      <c r="B12" s="17" t="inlineStr"/>
+      <c r="A12" s="14" t="inlineStr"/>
+      <c r="B12" s="15" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
       </c>
-      <c r="B13" s="17" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>docs/LegendaryTriggers.md, docs/LegendaryPlacementReview.md, data/totem_trials.yaml, decomp/res/field/events/*.json</t>
         </is>

</xml_diff>